<commit_message>
- Commit message for changes to pip package files in the .venv directory.
</commit_message>
<xml_diff>
--- a/Relatórios Recebidos/Relatorio de proprietarios.xlsx
+++ b/Relatórios Recebidos/Relatorio de proprietarios.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/53359c59c4c07b84/Documentos/Python Scripts/Projeto Metis/Relatórios Recebidos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="91" documentId="13_ncr:1_{E30B89C4-FCF1-4E57-A3EF-4E8A9712AD20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A59093C-C4FB-4FBA-9392-DE50651C14CE}"/>
+  <xr:revisionPtr revIDLastSave="96" documentId="13_ncr:1_{E30B89C4-FCF1-4E57-A3EF-4E8A9712AD20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01780AD0-9B20-4F0B-878F-CF698822393F}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="127" yWindow="150" windowWidth="19201" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Proprietarios" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId3"/>
+    <pivotCache cacheId="1" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -22729,7 +22729,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -22740,19 +22740,16 @@
       <b/>
       <sz val="8"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="8"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -22905,93 +22902,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="10079990" cy="0"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Shape 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="10079990" cy="0"/>
-        </a:xfrm>
-        <a:custGeom>
-          <a:avLst/>
-          <a:gdLst/>
-          <a:ahLst/>
-          <a:cxnLst/>
-          <a:rect l="0" t="0" r="0" b="0"/>
-          <a:pathLst>
-            <a:path w="10079990">
-              <a:moveTo>
-                <a:pt x="0" y="0"/>
-              </a:moveTo>
-              <a:lnTo>
-                <a:pt x="2597658" y="0"/>
-              </a:lnTo>
-            </a:path>
-            <a:path w="10079990">
-              <a:moveTo>
-                <a:pt x="2597658" y="0"/>
-              </a:moveTo>
-              <a:lnTo>
-                <a:pt x="3844797" y="0"/>
-              </a:lnTo>
-            </a:path>
-            <a:path w="10079990">
-              <a:moveTo>
-                <a:pt x="3844797" y="0"/>
-              </a:moveTo>
-              <a:lnTo>
-                <a:pt x="4884039" y="0"/>
-              </a:lnTo>
-            </a:path>
-            <a:path w="10079990">
-              <a:moveTo>
-                <a:pt x="4884039" y="0"/>
-              </a:moveTo>
-              <a:lnTo>
-                <a:pt x="7481824" y="0"/>
-              </a:lnTo>
-            </a:path>
-            <a:path w="10079990">
-              <a:moveTo>
-                <a:pt x="7481824" y="0"/>
-              </a:moveTo>
-              <a:lnTo>
-                <a:pt x="10079990" y="0"/>
-              </a:lnTo>
-            </a:path>
-          </a:pathLst>
-        </a:custGeom>
-        <a:ln w="10795">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -31074,7 +30984,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D1B14F51-05E3-4DF8-8345-4895745DCFDD}" name="Tabela dinâmica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D1B14F51-05E3-4DF8-8345-4895745DCFDD}" name="Tabela dinâmica2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:C671" firstHeaderRow="1" firstDataRow="1" firstDataCol="2"/>
   <pivotFields count="9">
     <pivotField compact="0" outline="0" showAll="0" defaultSubtotal="0"/>
@@ -57240,7 +57150,6 @@
     <hyperlink ref="E670" r:id="rId1100" display="mailto:zvonimir@zupan.com.br" xr:uid="{00000000-0004-0000-0000-00004C040000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1101"/>
 </worksheet>
 </file>
 

</xml_diff>